<commit_message>
feat: align ship slots and player defence survival
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/ship.xlsx
+++ b/space-battleship/config_excel/ship.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="12375" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ship" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ship" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1130,10 +1130,10 @@
         </is>
       </c>
       <c r="C4" s="0" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="0" t="n">
         <v>50</v>
@@ -1157,10 +1157,10 @@
         </is>
       </c>
       <c r="C5" s="0" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="0" t="n">
         <v>50</v>
@@ -1184,10 +1184,10 @@
         </is>
       </c>
       <c r="C6" s="0" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" s="0" t="n">
         <v>50</v>
@@ -1211,10 +1211,10 @@
         </is>
       </c>
       <c r="C7" s="0" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D7" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" s="0" t="n">
         <v>50</v>
@@ -1238,10 +1238,10 @@
         </is>
       </c>
       <c r="C8" s="0" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D8" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8" s="0" t="n">
         <v>50</v>

</xml_diff>